<commit_message>
feat(F-NAR-009): SEC.ADU/MAI/PAR/RUE, ramifiées COL-033–035 et DIF-001–013
Ouvertures monde d’abord, chacune différente. Audio plus tard.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-SEC.ADU.001-02.xlsx
+++ b/stories/arbres/ATOM-SEC.ADU.001-02.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hanna va vers maman, puis la maîtresse</t>
+          <t>Les yaourts et la main de papa</t>
         </is>
       </c>
     </row>
@@ -830,6 +830,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Les yaourts sont froids. Aniss cherche. Il va vers maman, puis vers la maîtresse, puis vers papa.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1184,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Hanna est au magasin. C'est après l'école. La maîtresse a dit au revoir près de la porte. Papa doit arriver plus tard. Maman pousse le panier. Hanna regarde les pots de yaourt. Ils sont frais. Elle lève les yeux. Elle cherche. Hanna se souvient. On va vers papa. On va vers maman. On va vers la maîtresse. Hanna marche vers les yaourts. Elle voit maman. Maman a le panier. Hanna va vers maman. Elle tient le manteau de maman. Ses pieds restent près de maman. Parce qu'elle a cherché maman, elle la trouve. Me voici. Le lendemain, Hanna est dans la cour. Elle cherche. Elle va vers la maîtresse. La maîtresse est près du bac. Hanna reste près de la maîtresse. Papa arrive. Hanna va vers papa. Elle prend la main de papa. Au magasin, puis à l'école, c'est pareil. On va vers papa, vers maman, ou vers la maîtresse.</t>
+          <t>Les pots de yaourt sont froids, tout ronds. Un pot a une petite étiquette bleue. Le rayon souffle un air frais. Ça sent le lait froid. Le sol du magasin brille, tout lisse. Un sac jaune froisse près du genou. La sangle du cartable laisse une marque tiède. Dehors, le jour baisse un peu. Une feuille sèche tourne près de la porte. Aniss vit avec papa et maman. C'est après l'école. La maîtresse a dit au revoir, près de la porte. Papa doit arriver plus tard. Aniss, tu vois les yaourts ? Oui, maman. Ils sont froids. On en prend deux ? Deux, oui. En ce moment, Aniss est au magasin. Maman pousse le panier. Le panier fait un petit couic. Aniss regarde les pots. Il lève les yeux. Il cherche. Maman ? Aniss se souvient. On va vers papa. On va vers maman. On va vers la maîtresse. Je vais vers maman. Aniss marche vers les yaourts. Ses pieds restent près du panier. Le sol est froid sous les chaussures. Il voit maman. Maman a le panier. Un pot blanc dépasse. Me voici, Aniss. Je t'ai cherchée. Tu vas vers papa, maman, ou la maîtresse. Bravo. Tu es venu vers maman. La maîtresse a dit au revoir. Oui. Papa arrive bientôt. Aniss va vers maman. Parce qu'il a cherché maman, il la trouve. Aniss tient le manteau de maman. Le manteau est laineux, un peu chaud. Il sent la maison. Tu as fait du bon travail. On reste ensemble. Le panier fait encore couic. Les pots restent froids. Le lendemain, la cour est claire. Le gravier craque sous les chaussures. Un bac à sable attend près du mur. Le vent pousse un peu de poussière. Aniss cherche. La maîtresse ? Il va vers la maîtresse. La maîtresse est près du bac. Aniss reste près de la maîtresse. Ses pieds restent près du bac. Papa arrive près du portail. Papa ! Aniss va vers papa. Il prend la main de papa. Me voici. Tu es venu vers moi ? Oui, papa. Vers papa. Bravo, Aniss. Tu vas vers papa, maman, ou la maîtresse. Au magasin, c'était pareil. C'est du bon travail. La main de papa est chaude. Le sac jaune sent encore le yaourt.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,14 +1324,88 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Hanna est au magasin. C'est après l'école. La maîtresse a dit au revoir près de la porte. Papa doit arriver plus tard. Maman pousse le panier. Hanna regarde les pots de yaourt. Ils sont frais. Elle lève les yeux. Elle cherche. Hanna se souvient. On va vers papa. On va vers maman. On va vers la maîtresse. Hanna marche vers les yaourts. Elle voit maman. Maman a le panier. Hanna va vers maman. Elle tient le manteau de maman. Ses pieds restent près de maman. Parce qu'elle a cherché maman, elle la trouve.
-maman|Me voici.
-narrateur|Le lendemain, Hanna est dans la cour. Elle cherche. Elle va vers la maîtresse. La maîtresse est près du bac. Hanna reste près de la maîtresse. Papa arrive. Hanna va vers papa. Elle prend la main de papa. Au magasin, puis à l'école, c'est pareil. On va vers papa, vers maman, ou vers la maîtresse.</t>
+          <t>narrateur|Les pots de yaourt sont froids, tout ronds.
+narrateur|Un pot a une petite étiquette bleue.
+narrateur|Le rayon souffle un air frais.
+narrateur|Ça sent le lait froid.
+narrateur|Le sol du magasin brille, tout lisse.
+narrateur|Un sac jaune froisse près du genou.
+narrateur|La sangle du cartable laisse une marque tiède.
+narrateur|Dehors, le jour baisse un peu.
+narrateur|Une feuille sèche tourne près de la porte.
+narrateur|Aniss vit avec papa et maman.
+narrateur|C'est après l'école.
+narrateur|La maîtresse a dit au revoir, près de la porte.
+narrateur|Papa doit arriver plus tard.
+maman|Aniss, tu vois les yaourts ?
+enfant-m|Oui, maman.
+enfant-m|Ils sont froids.
+maman|On en prend deux ?
+enfant-m|Deux, oui.
+narrateur|En ce moment, Aniss est au magasin.
+narrateur|Maman pousse le panier.
+narrateur|Le panier fait un petit couic.
+narrateur|Aniss regarde les pots.
+narrateur|Il lève les yeux.
+narrateur|Il cherche.
+enfant-m|Maman ?
+narrateur|Aniss se souvient.
+narrateur|On va vers papa.
+narrateur|On va vers maman.
+narrateur|On va vers la maîtresse.
+enfant-m|Je vais vers maman.
+narrateur|Aniss marche vers les yaourts.
+narrateur|Ses pieds restent près du panier.
+narrateur|Le sol est froid sous les chaussures.
+narrateur|Il voit maman.
+narrateur|Maman a le panier.
+narrateur|Un pot blanc dépasse.
+maman|Me voici, Aniss.
+enfant-m|Je t'ai cherchée.
+maman|Tu vas vers papa, maman, ou la maîtresse.
+maman|Bravo.
+maman|Tu es venu vers maman.
+enfant-m|La maîtresse a dit au revoir.
+maman|Oui.
+maman|Papa arrive bientôt.
+narrateur|Aniss va vers maman.
+narrateur|Parce qu'il a cherché maman, il la trouve.
+narrateur|Aniss tient le manteau de maman.
+narrateur|Le manteau est laineux, un peu chaud.
+enfant-m|Il sent la maison.
+maman|Tu as fait du bon travail.
+maman|On reste ensemble.
+narrateur|Le panier fait encore couic.
+narrateur|Les pots restent froids.
+narrateur|Le lendemain, la cour est claire.
+narrateur|Le gravier craque sous les chaussures.
+narrateur|Un bac à sable attend près du mur.
+narrateur|Le vent pousse un peu de poussière.
+narrateur|Aniss cherche.
+enfant-m|La maîtresse ?
+narrateur|Il va vers la maîtresse.
+narrateur|La maîtresse est près du bac.
+narrateur|Aniss reste près de la maîtresse.
+narrateur|Ses pieds restent près du bac.
+narrateur|Papa arrive près du portail.
+enfant-m|Papa !
+narrateur|Aniss va vers papa.
+narrateur|Il prend la main de papa.
+papa|Me voici.
+papa|Tu es venu vers moi ?
+enfant-m|Oui, papa.
+enfant-m|Vers papa.
+papa|Bravo, Aniss.
+papa|Tu vas vers papa, maman, ou la maîtresse.
+maman|Au magasin, c'était pareil.
+papa|C'est du bon travail.
+narrateur|La main de papa est chaude.
+narrateur|Le sac jaune sent encore le yaourt.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>caddie</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1432,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Hanna cherche quelqu'un. Vers qui va-t-elle ?</t>
+          <t>Aniss cherche quelqu'un. Vers qui va-t-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1506,7 +1592,8 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Hanna cherche quelqu'un. Vers qui va-t-elle ?</t>
+          <t>narrateur|Aniss cherche quelqu'un.
+narrateur|Vers qui va-t-il ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1534,7 +1621,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Hanna a cherché maman. À l'école, elle va vers la maîtresse. Papa est aussi un adulte connu.</t>
+          <t>Aniss a cherché maman. Il est allé vers maman. Tu es venu vers moi ? Oui. Vers maman. Bravo, Aniss. Papa et la maîtresse sont aussi des adultes connus. À l'école, il va vers la maîtresse. Et vers moi, aussi. Vers papa. Bravo. Aniss tient encore le manteau. Le manteau sent encore la maison.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1595,14 +1682,14 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
         <v>0.96</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1682,7 +1769,19 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Hanna a cherché maman. À l'école, elle va vers la maîtresse. Papa est aussi un adulte connu.</t>
+          <t>narrateur|Aniss a cherché maman.
+narrateur|Il est allé vers maman.
+maman|Tu es venu vers moi ?
+enfant-m|Oui.
+enfant-m|Vers maman.
+maman|Bravo, Aniss.
+maman|Papa et la maîtresse sont aussi des adultes connus.
+narrateur|À l'école, il va vers la maîtresse.
+papa|Et vers moi, aussi.
+enfant-m|Vers papa.
+papa|Bravo.
+narrateur|Aniss tient encore le manteau.
+narrateur|Le manteau sent encore la maison.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1710,7 +1809,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Hanna tient la main de papa. Ils rentrent.</t>
+          <t>Papa tient la main d'Aniss. On rentre ? Oui, papa. Tu as fini ? Oui. Le sac sent le yaourt. Merci, maman. Merci, papa. Merci, Aniss. Tu vas vers papa, maman, ou la maîtresse. Bravo. Ils passent près du portail. Le gravier craque encore. Le yaourt reste froid, dans le sac.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1771,14 +1870,14 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
         <v>0.96</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1854,7 +1953,20 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Hanna tient la main de papa. Ils rentrent.</t>
+          <t>narrateur|Papa tient la main d'Aniss.
+papa|On rentre ?
+enfant-m|Oui, papa.
+papa|Tu as fini ?
+enfant-m|Oui.
+maman|Le sac sent le yaourt.
+enfant-m|Merci, maman.
+enfant-m|Merci, papa.
+papa|Merci, Aniss.
+maman|Tu vas vers papa, maman, ou la maîtresse.
+papa|Bravo.
+narrateur|Ils passent près du portail.
+narrateur|Le gravier craque encore.
+narrateur|Le yaourt reste froid, dans le sac.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1882,7 +1994,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Je suis allé vers maman. Puis vers la maîtresse. Puis vers papa. Bravo. Tu as fait du bon travail. Le sac sent encore le yaourt. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1943,14 +2055,14 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
         <v>0.92</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2022,7 +2134,13 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>enfant-m|Je suis allé vers maman.
+enfant-m|Puis vers la maîtresse.
+enfant-m|Puis vers papa.
+maman|Bravo.
+papa|Tu as fait du bon travail.
+narrateur|Le sac sent encore le yaourt.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2044,7 +2162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2082,6 +2200,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>